<commit_message>
builds and validates test .xml
</commit_message>
<xml_diff>
--- a/create_xml_R/data-raw/metadata/results_metadata.xlsx
+++ b/create_xml_R/data-raw/metadata/results_metadata.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Liz/Documents/code/JPE/jpe-genetics-edi/create_xml_R/data-raw/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Liz/Documents/code/JPE/jpe-genetics-edi/create_xml_R/data-raw/metadata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{021215EB-EFF7-0E4A-826F-27DD0148365F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{429037C2-8413-3340-B2F1-5E2E97B38323}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="2100" windowWidth="30240" windowHeight="17200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1212,8 +1212,12 @@
       <c r="I15" s="5"/>
       <c r="J15" s="6"/>
       <c r="K15" s="5"/>
-      <c r="L15" s="6"/>
-      <c r="M15" s="6"/>
+      <c r="L15" s="6">
+        <v>0</v>
+      </c>
+      <c r="M15" s="6">
+        <v>1</v>
+      </c>
       <c r="N15" s="4"/>
       <c r="O15" s="4"/>
       <c r="P15" s="4"/>

</xml_diff>